<commit_message>
Changed data, and added timing for the heuristic
</commit_message>
<xml_diff>
--- a/inputData/Experiments/inputDataEx5_3_10.xlsx
+++ b/inputData/Experiments/inputDataEx5_3_10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22DA0F23-2D6B-421A-84A5-DC5A87FB507F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF842D8-998C-42AD-B42C-17E0A8FB7F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="8170" activeTab="2" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="PlaneData" sheetId="7" r:id="rId1"/>
@@ -820,7 +820,7 @@
         <v>35</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -900,7 +900,7 @@
         <v>50</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11">
         <v>1</v>

</xml_diff>